<commit_message>
Redesigned to use clone accelerometer module
</commit_message>
<xml_diff>
--- a/design/production/design-all-pos.xlsx
+++ b/design/production/design-all-pos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Felix\Documents\GameDev\multifunctional-fn-keyboard\design\production\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2BDB3A24-08D0-479F-84F5-547D41638381}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B0184D10-933B-4B3B-AFA7-DFC3D59A2AED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{AD8CC6E5-7FA0-4ACC-8039-0FD99978465B}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11385" xr2:uid="{90EF1357-435D-4D50-B57E-B1145F3879A7}"/>
   </bookViews>
   <sheets>
     <sheet name="design-all-pos" sheetId="1" r:id="rId1"/>
@@ -150,19 +150,19 @@
     <t>U1</t>
   </si>
   <si>
-    <t>LSM6DS3</t>
-  </si>
-  <si>
-    <t>LGA-14_3x2.5mm_P0.5mm_LayoutBorder3x4y</t>
+    <t>RaspberryPi_Pico</t>
+  </si>
+  <si>
+    <t>RaspberryPi_Pico_Common_Unspecified</t>
   </si>
   <si>
     <t>U2</t>
   </si>
   <si>
-    <t>RaspberryPi_Pico</t>
-  </si>
-  <si>
-    <t>RaspberryPi_Pico_Common_Unspecified</t>
+    <t>LIS2DW12</t>
+  </si>
+  <si>
+    <t>LGA12R50P4X4_200X200X70</t>
   </si>
   <si>
     <t>Designator</t>
@@ -1034,14 +1034,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBACFEE8-3AE2-483A-AC39-6E765A61D89F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6549848-91C8-4991-B8E6-306CF231E946}">
   <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="20.140625" customWidth="1"/>
-    <col min="2" max="2" width="32.7109375" customWidth="1"/>
-    <col min="3" max="3" width="25" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -1077,10 +1072,10 @@
         <v>5</v>
       </c>
       <c r="D2">
-        <v>166.38</v>
+        <v>168.62</v>
       </c>
       <c r="E2">
-        <v>-88.9</v>
+        <v>-91.7</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1100,13 +1095,13 @@
         <v>5</v>
       </c>
       <c r="D3">
-        <v>166.28</v>
+        <v>168.3</v>
       </c>
       <c r="E3">
-        <v>-91.4</v>
+        <v>-90.3</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="G3" t="s">
         <v>6</v>
@@ -1583,13 +1578,13 @@
         <v>42</v>
       </c>
       <c r="D24">
-        <v>163.41249999999999</v>
+        <v>137.75</v>
       </c>
       <c r="E24">
-        <v>-90.9</v>
+        <v>-84.1</v>
       </c>
       <c r="F24">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="G24" t="s">
         <v>6</v>
@@ -1606,10 +1601,10 @@
         <v>45</v>
       </c>
       <c r="D25">
-        <v>137.75</v>
+        <v>165.76249999999999</v>
       </c>
       <c r="E25">
-        <v>-84.1</v>
+        <v>-91.7</v>
       </c>
       <c r="F25">
         <v>0</v>

</xml_diff>